<commit_message>
feat(uncertainty): 65-band DIAS MultiCP & SCMCP 3-model re-computation, realigned notebooks, publication docx reports
</commit_message>
<xml_diff>
--- a/dapm/results/dapm_full_reports_all_models.xlsx
+++ b/dapm/results/dapm_full_reports_all_models.xlsx
@@ -163,7 +163,7 @@
     <t>['AlexNet_CNN', 'GFNet', 'ViT_UNet']</t>
   </si>
   <si>
-    <t>2026-10-12T06:10:54.331205+00:00</t>
+    <t>2026-10-23T07:41:00.680963+00:00</t>
   </si>
   <si>
     <t>class_id</t>
@@ -1778,7 +1778,7 @@
         <v>0.1613004505634308</v>
       </c>
       <c r="M2">
-        <v>464.7843692302704</v>
+        <v>486.6822035312653</v>
       </c>
       <c r="N2">
         <v>0.9992162982280177</v>
@@ -1825,7 +1825,7 @@
         <v>0.1648713499307632</v>
       </c>
       <c r="M3">
-        <v>500.4662084579468</v>
+        <v>518.1863608360291</v>
       </c>
       <c r="N3">
         <v>0.9999447879858657</v>
@@ -1872,7 +1872,7 @@
         <v>0.1709258407354355</v>
       </c>
       <c r="M4">
-        <v>533.3799152374268</v>
+        <v>542.1092395782471</v>
       </c>
       <c r="N4">
         <v>0.9994400142158111</v>
@@ -2811,7 +2811,7 @@
         <v>0.1613004505634308</v>
       </c>
       <c r="M5">
-        <v>464.7843692302704</v>
+        <v>486.6822035312653</v>
       </c>
       <c r="N5">
         <v>0.9992162982280177</v>
@@ -3307,7 +3307,7 @@
         <v>0.1648713499307632</v>
       </c>
       <c r="M5">
-        <v>500.4662084579468</v>
+        <v>518.1863608360291</v>
       </c>
       <c r="N5">
         <v>0.9999447879858657</v>
@@ -3803,7 +3803,7 @@
         <v>0.1709258407354355</v>
       </c>
       <c r="M5">
-        <v>533.3799152374268</v>
+        <v>542.1092395782471</v>
       </c>
       <c r="N5">
         <v>0.9994400142158111</v>
@@ -4291,7 +4291,7 @@
         <v>0.1613004505634308</v>
       </c>
       <c r="M4">
-        <v>464.7843692302704</v>
+        <v>486.6822035312653</v>
       </c>
       <c r="N4">
         <v>0.9992162982280177</v>
@@ -4338,7 +4338,7 @@
         <v>0.1648713499307632</v>
       </c>
       <c r="M5">
-        <v>500.4662084579468</v>
+        <v>518.1863608360291</v>
       </c>
       <c r="N5">
         <v>0.9999447879858657</v>
@@ -4385,7 +4385,7 @@
         <v>0.1709258407354355</v>
       </c>
       <c r="M6">
-        <v>533.3799152374268</v>
+        <v>542.1092395782471</v>
       </c>
       <c r="N6">
         <v>0.9994400142158111</v>

</xml_diff>